<commit_message>
lookup file changed and months blank removed
</commit_message>
<xml_diff>
--- a/lookup.xlsx
+++ b/lookup.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2194998_cognizant_com/Documents/Desktop/Final_RES AI PRO_All Done 1/Final_RES AI PRO_All Done/python_automation_utility/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2194998_cognizant_com/Documents/Desktop/AutoOptix_V2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{8DED2FE9-96A2-42D0-9AE4-5080708F5C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="14_{8DED2FE9-96A2-42D0-9AE4-5080708F5C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4A09A53-5C3A-4F49-AF4D-EBC2939F7063}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0A1DFA8F-19F2-4D04-A498-FC5F4A4BC30D}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$676</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3998" uniqueCount="765">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4055" uniqueCount="779">
   <si>
     <t>Subgroup</t>
   </si>
@@ -2334,6 +2334,48 @@
   </si>
   <si>
     <t>non-actionable</t>
+  </si>
+  <si>
+    <t>PagerDuty</t>
+  </si>
+  <si>
+    <t>Datadog</t>
+  </si>
+  <si>
+    <t>Termination</t>
+  </si>
+  <si>
+    <t>Contingent Worker</t>
+  </si>
+  <si>
+    <t>Onboarding/Offboarding Request</t>
+  </si>
+  <si>
+    <t>Sharepoint</t>
+  </si>
+  <si>
+    <t>Sharepoint Access</t>
+  </si>
+  <si>
+    <t>Ecom Order</t>
+  </si>
+  <si>
+    <t>Splunk Alert</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>L2</t>
   </si>
 </sst>
 </file>
@@ -2409,7 +2451,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2425,6 +2467,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2761,15 +2806,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3556B986-2304-4B99-95C9-14CF88AE4CEB}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H676"/>
+  <dimension ref="A1:I691"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.08984375" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" customWidth="1"/>
     <col min="2" max="2" width="32.7265625" customWidth="1"/>
     <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="106.81640625" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -19442,7 +19487,7 @@
         <v>L1.5</v>
       </c>
     </row>
-    <row r="673" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="673" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A673" s="7" t="s">
         <v>761</v>
       </c>
@@ -19464,7 +19509,7 @@
         <v>L1.5</v>
       </c>
     </row>
-    <row r="674" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="674" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A674" s="7" t="s">
         <v>762</v>
       </c>
@@ -19486,7 +19531,7 @@
         <v>L1.5</v>
       </c>
     </row>
-    <row r="675" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="675" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A675" s="7" t="s">
         <v>763</v>
       </c>
@@ -19508,7 +19553,7 @@
         <v>L1.5</v>
       </c>
     </row>
-    <row r="676" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="676" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A676" s="7" t="s">
         <v>764</v>
       </c>
@@ -19529,6 +19574,270 @@
         <f t="shared" si="10"/>
         <v>L1.5</v>
       </c>
+    </row>
+    <row r="677" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A677" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="B677" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C677" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="D677" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F677" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="G677" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="H677" s="8" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="678" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A678" s="3" t="s">
+        <v>766</v>
+      </c>
+      <c r="B678" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C678" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="D678" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F678" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="G678" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="H678" s="8" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="679" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A679" s="3" t="s">
+        <v>767</v>
+      </c>
+      <c r="B679" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="C679" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="D679" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F679" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="G679" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="H679" s="8" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="680" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A680" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="B680" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="C680" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="D680" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F680" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="G680" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="H680" s="8" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="681" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A681" s="3" t="s">
+        <v>770</v>
+      </c>
+      <c r="B681" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="C681" s="8"/>
+      <c r="D681" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F681" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="G681" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="H681" s="8" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="682" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A682" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="B682" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C682" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="D682" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F682" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="G682" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="H682" s="8" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="683" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A683" s="3" t="s">
+        <v>772</v>
+      </c>
+      <c r="B683" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C683" s="8" t="s">
+        <v>777</v>
+      </c>
+      <c r="D683" s="8" t="s">
+        <v>777</v>
+      </c>
+      <c r="E683" s="8" t="s">
+        <v>777</v>
+      </c>
+      <c r="F683" s="8" t="s">
+        <v>777</v>
+      </c>
+      <c r="G683" s="8" t="s">
+        <v>777</v>
+      </c>
+      <c r="H683" s="8" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="684" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A684" s="1"/>
+      <c r="B684" s="1"/>
+      <c r="C684" s="1"/>
+      <c r="D684" s="1"/>
+      <c r="E684" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F684" s="2"/>
+      <c r="G684" s="2"/>
+    </row>
+    <row r="685" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A685" s="8"/>
+      <c r="B685" s="8"/>
+      <c r="C685" s="8"/>
+      <c r="D685" s="8"/>
+      <c r="E685" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="F685" s="8"/>
+      <c r="G685" s="8"/>
+      <c r="H685" s="8"/>
+      <c r="I685" s="8"/>
+    </row>
+    <row r="686" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A686" s="8"/>
+      <c r="B686" s="8"/>
+      <c r="C686" s="8"/>
+      <c r="D686" s="8"/>
+      <c r="E686" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="F686" s="8"/>
+      <c r="G686" s="8"/>
+      <c r="H686" s="8"/>
+      <c r="I686" s="8"/>
+    </row>
+    <row r="687" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A687" s="8"/>
+      <c r="B687" s="8"/>
+      <c r="C687" s="8"/>
+      <c r="D687" s="8"/>
+      <c r="E687" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="F687" s="8"/>
+      <c r="G687" s="8"/>
+      <c r="H687" s="8"/>
+      <c r="I687" s="8"/>
+    </row>
+    <row r="688" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A688" s="8"/>
+      <c r="B688" s="8"/>
+      <c r="C688" s="8"/>
+      <c r="D688" s="8"/>
+      <c r="E688" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="F688" s="8"/>
+      <c r="G688" s="8"/>
+      <c r="H688" s="8"/>
+      <c r="I688" s="8"/>
+    </row>
+    <row r="689" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A689" s="8"/>
+      <c r="B689" s="8"/>
+      <c r="C689" s="8"/>
+      <c r="D689" s="8"/>
+      <c r="E689" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="F689" s="8"/>
+      <c r="G689" s="8"/>
+      <c r="H689" s="8"/>
+      <c r="I689" s="8"/>
+    </row>
+    <row r="690" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A690" s="8"/>
+      <c r="B690" s="8"/>
+      <c r="C690" s="8"/>
+      <c r="D690" s="8"/>
+      <c r="E690" s="8" t="s">
+        <v>774</v>
+      </c>
+      <c r="F690" s="8"/>
+      <c r="G690" s="8"/>
+      <c r="H690" s="8"/>
+      <c r="I690" s="8"/>
+    </row>
+    <row r="691" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A691" s="8"/>
+      <c r="B691" s="8"/>
+      <c r="C691" s="8"/>
+      <c r="D691" s="8"/>
+      <c r="E691" s="8" t="s">
+        <v>777</v>
+      </c>
+      <c r="F691" s="8"/>
+      <c r="G691" s="8"/>
+      <c r="H691" s="8"/>
+      <c r="I691" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H676" xr:uid="{F2B32AB8-7948-4E69-AD33-69BDDAAC2B40}">

</xml_diff>